<commit_message>
done week 4 & 5
</commit_message>
<xml_diff>
--- a/SWP391_SE20A07_DE190512_MaiVanLuong.xlsx
+++ b/SWP391_SE20A07_DE190512_MaiVanLuong.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SU26\SWP\audit-log\swp391-aiauditlog-MaiLuong1906\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{373AF627-CF90-4F0F-8A83-B94BAD58AE74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38AD4DA3-D688-4962-824D-09030DF9ECF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1312,13 +1312,22 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1327,15 +1336,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1650,14 +1650,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="29" t="s">
         <v>152</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -1875,7 +1875,7 @@
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="4" max="4" width="25.5" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="35" customWidth="1"/>
     <col min="7" max="7" width="50" customWidth="1"/>
@@ -1883,28 +1883,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
     </row>
     <row r="3" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
@@ -2521,22 +2521,22 @@
       </c>
     </row>
     <row r="27" spans="1:8" ht="59.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="31">
+      <c r="A27" s="25">
         <v>24</v>
       </c>
-      <c r="B27" s="31" t="s">
+      <c r="B27" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="C27" s="31" t="s">
+      <c r="C27" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="D27" s="31" t="s">
+      <c r="D27" s="25" t="s">
         <v>127</v>
       </c>
-      <c r="E27" s="31" t="s">
+      <c r="E27" s="25" t="s">
         <v>128</v>
       </c>
-      <c r="F27" s="31" t="s">
+      <c r="F27" s="25" t="s">
         <v>129</v>
       </c>
       <c r="G27" s="20" t="s">
@@ -2547,22 +2547,22 @@
       </c>
     </row>
     <row r="28" spans="1:8" ht="103.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="31">
+      <c r="A28" s="25">
         <v>25</v>
       </c>
-      <c r="B28" s="31" t="s">
+      <c r="B28" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="C28" s="31" t="s">
+      <c r="C28" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="D28" s="31" t="s">
+      <c r="D28" s="25" t="s">
         <v>132</v>
       </c>
-      <c r="E28" s="31" t="s">
+      <c r="E28" s="25" t="s">
         <v>133</v>
       </c>
-      <c r="F28" s="31" t="s">
+      <c r="F28" s="25" t="s">
         <v>134</v>
       </c>
       <c r="G28" s="20" t="s">
@@ -2573,22 +2573,22 @@
       </c>
     </row>
     <row r="29" spans="1:8" ht="234.6" x14ac:dyDescent="0.25">
-      <c r="A29" s="31">
+      <c r="A29" s="25">
         <v>26</v>
       </c>
-      <c r="B29" s="31" t="s">
+      <c r="B29" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="C29" s="31" t="s">
+      <c r="C29" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="D29" s="31" t="s">
+      <c r="D29" s="25" t="s">
         <v>137</v>
       </c>
-      <c r="E29" s="31" t="s">
+      <c r="E29" s="25" t="s">
         <v>138</v>
       </c>
-      <c r="F29" s="31" t="s">
+      <c r="F29" s="25" t="s">
         <v>139</v>
       </c>
       <c r="G29" s="20" t="s">
@@ -2599,22 +2599,22 @@
       </c>
     </row>
     <row r="30" spans="1:8" ht="220.8" x14ac:dyDescent="0.25">
-      <c r="A30" s="31">
+      <c r="A30" s="25">
         <v>27</v>
       </c>
-      <c r="B30" s="31" t="s">
+      <c r="B30" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="C30" s="31" t="s">
+      <c r="C30" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="D30" s="31" t="s">
+      <c r="D30" s="25" t="s">
         <v>142</v>
       </c>
-      <c r="E30" s="31" t="s">
+      <c r="E30" s="25" t="s">
         <v>143</v>
       </c>
-      <c r="F30" s="31" t="s">
+      <c r="F30" s="25" t="s">
         <v>144</v>
       </c>
       <c r="G30" s="20" t="s">
@@ -2625,22 +2625,22 @@
       </c>
     </row>
     <row r="31" spans="1:8" ht="234.6" x14ac:dyDescent="0.25">
-      <c r="A31" s="31">
+      <c r="A31" s="25">
         <v>28</v>
       </c>
-      <c r="B31" s="31" t="s">
+      <c r="B31" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="C31" s="31" t="s">
+      <c r="C31" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="D31" s="31" t="s">
+      <c r="D31" s="25" t="s">
         <v>147</v>
       </c>
-      <c r="E31" s="31" t="s">
+      <c r="E31" s="25" t="s">
         <v>148</v>
       </c>
-      <c r="F31" s="31" t="s">
+      <c r="F31" s="25" t="s">
         <v>149</v>
       </c>
       <c r="G31" s="20" t="s">
@@ -2671,24 +2671,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="32" t="s">
         <v>188</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="31" t="s">
         <v>189</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -3066,20 +3066,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="29" t="s">
         <v>248</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="33" t="s">
         <v>249</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
     </row>
     <row r="4" spans="1:4" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">

</xml_diff>